<commit_message>
Add student and class to workbook title
</commit_message>
<xml_diff>
--- a/Design_de_teste_Tarefa_2.xlsx
+++ b/Design_de_teste_Tarefa_2.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes de equivalência" sheetId="1" r:id="Rfa0dac404d7147c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de teste" sheetId="2" r:id="R9949ef62a7cf4965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes de equivalência" sheetId="1" r:id="Rb0d98234d3804b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de teste" sheetId="2" r:id="R831b2515cfd24a15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -488,7 +488,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>Projeto para GitHub: Design de teste - Tarefa 2 | Título acadêmico: nome, sobrenome e grupo pendentes | 2º sprint</x:v>
+        <x:v>Rafael Reis - Turma 30 - Projeto Design de teste - 2º sprint</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1404,7 +1404,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
-        <x:v>Projeto para GitHub: Design de teste - Tarefa 2 | Título acadêmico: nome, sobrenome e grupo pendentes | 2º sprint</x:v>
+        <x:v>Rafael Reis - Turma 30 - Projeto Design de teste - 2º sprint</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>

</xml_diff>